<commit_message>
Registers run inside the pipeline; the site deploys by command
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brazil/FINAL_PANEL.xlsx
+++ b/brazil/FINAL_PANEL.xlsx
@@ -1295,7 +1295,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>improving</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -2925,7 +2925,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>improving</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -3965,7 +3965,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>improving</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -7323,7 +7323,7 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
@@ -10088,7 +10088,7 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
@@ -15805,7 +15805,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>improving</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -17060,7 +17060,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>improving</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -17850,7 +17850,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>improving</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -20428,7 +20428,7 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
@@ -22568,7 +22568,7 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">

</xml_diff>

<commit_message>
Add brazil, brunei, thailand to the dashboard
</commit_message>
<xml_diff>
--- a/brazil/FINAL_PANEL.xlsx
+++ b/brazil/FINAL_PANEL.xlsx
@@ -1069,7 +1069,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>improving</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -2925,7 +2925,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>improving</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -3965,7 +3965,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>improving</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -8639,7 +8639,7 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
@@ -10088,7 +10088,7 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
@@ -15629,7 +15629,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -15805,7 +15805,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>improving</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -16972,7 +16972,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -17060,7 +17060,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>improving</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -17850,7 +17850,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>improving</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -21444,7 +21444,7 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
@@ -22568,7 +22568,7 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">

</xml_diff>

<commit_message>
Maldives withheld pending a readable parse; head capacity, config and handoff checks
</commit_message>
<xml_diff>
--- a/brazil/FINAL_PANEL.xlsx
+++ b/brazil/FINAL_PANEL.xlsx
@@ -4600,7 +4600,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>improving</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -5896,7 +5896,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>improving</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -6254,7 +6254,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>improving</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -6607,7 +6607,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>improving</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
@@ -7777,7 +7777,7 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>improving</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
@@ -8140,7 +8140,7 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>improving</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
@@ -8967,7 +8967,7 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>improving</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
@@ -9809,7 +9809,7 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>improving</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
@@ -15104,7 +15104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15125,20 +15125,30 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>printed_total</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>total_basis</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>matched_amount</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>coverage_pct</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>programs_matched</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>programs_total</t>
         </is>
@@ -15161,13 +15171,21 @@
       <c r="D2" t="n">
         <v>0</v>
       </c>
-      <c r="E2" t="n">
-        <v>0</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -15183,19 +15201,27 @@
         </is>
       </c>
       <c r="C3" t="n">
+        <v>947.5</v>
+      </c>
+      <c r="D3" t="n">
         <v>947.481</v>
       </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -15210,18 +15236,26 @@
         </is>
       </c>
       <c r="C4" t="n">
+        <v>32101.8</v>
+      </c>
+      <c r="D4" t="n">
         <v>32101.792</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
         <v>31837.4</v>
       </c>
-      <c r="E4" t="n">
+      <c r="G4" t="n">
         <v>99.2</v>
       </c>
-      <c r="F4" t="n">
+      <c r="H4" t="n">
         <v>10</v>
       </c>
-      <c r="G4" t="n">
+      <c r="I4" t="n">
         <v>15</v>
       </c>
     </row>
@@ -15237,18 +15271,26 @@
         </is>
       </c>
       <c r="C5" t="n">
+        <v>92730.7</v>
+      </c>
+      <c r="D5" t="n">
         <v>92730.663</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
         <v>14900.5</v>
       </c>
-      <c r="E5" t="n">
+      <c r="G5" t="n">
         <v>16.1</v>
       </c>
-      <c r="F5" t="n">
+      <c r="H5" t="n">
         <v>2</v>
       </c>
-      <c r="G5" t="n">
+      <c r="I5" t="n">
         <v>5</v>
       </c>
     </row>
@@ -15264,18 +15306,26 @@
         </is>
       </c>
       <c r="C6" t="n">
+        <v>16664.3</v>
+      </c>
+      <c r="D6" t="n">
         <v>16664.296</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
         <v>5415.6</v>
       </c>
-      <c r="E6" t="n">
+      <c r="G6" t="n">
         <v>32.5</v>
       </c>
-      <c r="F6" t="n">
+      <c r="H6" t="n">
         <v>2</v>
       </c>
-      <c r="G6" t="n">
+      <c r="I6" t="n">
         <v>4</v>
       </c>
     </row>
@@ -15291,18 +15341,26 @@
         </is>
       </c>
       <c r="C7" t="n">
+        <v>4135.5</v>
+      </c>
+      <c r="D7" t="n">
         <v>4135.507</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
         <v>1125</v>
       </c>
-      <c r="E7" t="n">
+      <c r="G7" t="n">
         <v>27.2</v>
       </c>
-      <c r="F7" t="n">
+      <c r="H7" t="n">
         <v>1</v>
       </c>
-      <c r="G7" t="n">
+      <c r="I7" t="n">
         <v>3</v>
       </c>
     </row>
@@ -15318,18 +15376,26 @@
         </is>
       </c>
       <c r="C8" t="n">
+        <v>278581.5</v>
+      </c>
+      <c r="D8" t="n">
         <v>278581.467</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
         <v>277724.3</v>
       </c>
-      <c r="E8" t="n">
+      <c r="G8" t="n">
         <v>99.7</v>
       </c>
-      <c r="F8" t="n">
+      <c r="H8" t="n">
         <v>7</v>
       </c>
-      <c r="G8" t="n">
+      <c r="I8" t="n">
         <v>9</v>
       </c>
     </row>
@@ -15345,18 +15411,26 @@
         </is>
       </c>
       <c r="C9" t="n">
+        <v>1002681.6</v>
+      </c>
+      <c r="D9" t="n">
         <v>1002681.586</v>
       </c>
-      <c r="D9" t="n">
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
         <v>886652.4</v>
       </c>
-      <c r="E9" t="n">
+      <c r="G9" t="n">
         <v>88.40000000000001</v>
       </c>
-      <c r="F9" t="n">
+      <c r="H9" t="n">
         <v>1</v>
       </c>
-      <c r="G9" t="n">
+      <c r="I9" t="n">
         <v>3</v>
       </c>
     </row>
@@ -15372,18 +15446,26 @@
         </is>
       </c>
       <c r="C10" t="n">
+        <v>219826.8</v>
+      </c>
+      <c r="D10" t="n">
         <v>219826.755</v>
       </c>
-      <c r="D10" t="n">
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
         <v>208505.3</v>
       </c>
-      <c r="E10" t="n">
+      <c r="G10" t="n">
         <v>94.8</v>
       </c>
-      <c r="F10" t="n">
+      <c r="H10" t="n">
         <v>7</v>
       </c>
-      <c r="G10" t="n">
+      <c r="I10" t="n">
         <v>11</v>
       </c>
     </row>
@@ -15399,18 +15481,26 @@
         </is>
       </c>
       <c r="C11" t="n">
+        <v>107634.1</v>
+      </c>
+      <c r="D11" t="n">
         <v>107634.125</v>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
         <v>78626.2</v>
       </c>
-      <c r="E11" t="n">
+      <c r="G11" t="n">
         <v>73</v>
       </c>
-      <c r="F11" t="n">
+      <c r="H11" t="n">
         <v>2</v>
       </c>
-      <c r="G11" t="n">
+      <c r="I11" t="n">
         <v>5</v>
       </c>
     </row>
@@ -15426,18 +15516,26 @@
         </is>
       </c>
       <c r="C12" t="n">
+        <v>162614</v>
+      </c>
+      <c r="D12" t="n">
         <v>162614.024</v>
       </c>
-      <c r="D12" t="n">
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
         <v>86971.7</v>
       </c>
-      <c r="E12" t="n">
+      <c r="G12" t="n">
         <v>53.5</v>
       </c>
-      <c r="F12" t="n">
+      <c r="H12" t="n">
         <v>3</v>
       </c>
-      <c r="G12" t="n">
+      <c r="I12" t="n">
         <v>6</v>
       </c>
     </row>
@@ -15453,18 +15551,26 @@
         </is>
       </c>
       <c r="C13" t="n">
+        <v>2877.3</v>
+      </c>
+      <c r="D13" t="n">
         <v>2877.345</v>
       </c>
-      <c r="D13" t="n">
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
         <v>2026.6</v>
       </c>
-      <c r="E13" t="n">
+      <c r="G13" t="n">
         <v>70.40000000000001</v>
       </c>
-      <c r="F13" t="n">
+      <c r="H13" t="n">
         <v>1</v>
       </c>
-      <c r="G13" t="n">
+      <c r="I13" t="n">
         <v>2</v>
       </c>
     </row>
@@ -15480,18 +15586,26 @@
         </is>
       </c>
       <c r="C14" t="n">
+        <v>2170.6</v>
+      </c>
+      <c r="D14" t="n">
         <v>2170.599</v>
       </c>
-      <c r="D14" t="n">
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
         <v>1412.4</v>
       </c>
-      <c r="E14" t="n">
+      <c r="G14" t="n">
         <v>65.09999999999999</v>
       </c>
-      <c r="F14" t="n">
+      <c r="H14" t="n">
         <v>17</v>
       </c>
-      <c r="G14" t="n">
+      <c r="I14" t="n">
         <v>21</v>
       </c>
     </row>
@@ -15507,18 +15621,26 @@
         </is>
       </c>
       <c r="C15" t="n">
+        <v>10239.4</v>
+      </c>
+      <c r="D15" t="n">
         <v>10239.386</v>
       </c>
-      <c r="D15" t="n">
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
         <v>9046.700000000001</v>
       </c>
-      <c r="E15" t="n">
+      <c r="G15" t="n">
         <v>88.40000000000001</v>
       </c>
-      <c r="F15" t="n">
+      <c r="H15" t="n">
         <v>6</v>
       </c>
-      <c r="G15" t="n">
+      <c r="I15" t="n">
         <v>7</v>
       </c>
     </row>
@@ -15534,18 +15656,26 @@
         </is>
       </c>
       <c r="C16" t="n">
+        <v>682.6</v>
+      </c>
+      <c r="D16" t="n">
         <v>682.617</v>
       </c>
-      <c r="D16" t="n">
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
         <v>682.6</v>
       </c>
-      <c r="E16" t="n">
+      <c r="G16" t="n">
         <v>100</v>
       </c>
-      <c r="F16" t="n">
+      <c r="H16" t="n">
         <v>2</v>
       </c>
-      <c r="G16" t="n">
+      <c r="I16" t="n">
         <v>2</v>
       </c>
     </row>
@@ -15561,18 +15691,26 @@
         </is>
       </c>
       <c r="C17" t="n">
+        <v>2937.2</v>
+      </c>
+      <c r="D17" t="n">
         <v>2937.235</v>
       </c>
-      <c r="D17" t="n">
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
         <v>2495.5</v>
       </c>
-      <c r="E17" t="n">
+      <c r="G17" t="n">
         <v>85</v>
       </c>
-      <c r="F17" t="n">
+      <c r="H17" t="n">
         <v>2</v>
       </c>
-      <c r="G17" t="n">
+      <c r="I17" t="n">
         <v>3</v>
       </c>
     </row>
@@ -15588,18 +15726,26 @@
         </is>
       </c>
       <c r="C18" t="n">
+        <v>15386.2</v>
+      </c>
+      <c r="D18" t="n">
         <v>15386.176</v>
       </c>
-      <c r="D18" t="n">
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
         <v>13557.4</v>
       </c>
-      <c r="E18" t="n">
+      <c r="G18" t="n">
         <v>88.09999999999999</v>
       </c>
-      <c r="F18" t="n">
+      <c r="H18" t="n">
         <v>6</v>
       </c>
-      <c r="G18" t="n">
+      <c r="I18" t="n">
         <v>9</v>
       </c>
     </row>
@@ -15615,18 +15761,26 @@
         </is>
       </c>
       <c r="C19" t="n">
+        <v>17427.2</v>
+      </c>
+      <c r="D19" t="n">
         <v>17427.157</v>
       </c>
-      <c r="D19" t="n">
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
         <v>6203.7</v>
       </c>
-      <c r="E19" t="n">
+      <c r="G19" t="n">
         <v>35.6</v>
       </c>
-      <c r="F19" t="n">
+      <c r="H19" t="n">
         <v>3</v>
       </c>
-      <c r="G19" t="n">
+      <c r="I19" t="n">
         <v>13</v>
       </c>
     </row>
@@ -15642,18 +15796,26 @@
         </is>
       </c>
       <c r="C20" t="n">
+        <v>29160.4</v>
+      </c>
+      <c r="D20" t="n">
         <v>29160.377</v>
       </c>
-      <c r="D20" t="n">
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
         <v>23107.1</v>
       </c>
-      <c r="E20" t="n">
+      <c r="G20" t="n">
         <v>79.2</v>
       </c>
-      <c r="F20" t="n">
+      <c r="H20" t="n">
         <v>8</v>
       </c>
-      <c r="G20" t="n">
+      <c r="I20" t="n">
         <v>10</v>
       </c>
     </row>
@@ -15669,18 +15831,26 @@
         </is>
       </c>
       <c r="C21" t="n">
+        <v>3304.9</v>
+      </c>
+      <c r="D21" t="n">
         <v>3304.874</v>
       </c>
-      <c r="D21" t="n">
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
         <v>592.4</v>
       </c>
-      <c r="E21" t="n">
+      <c r="G21" t="n">
         <v>17.9</v>
       </c>
-      <c r="F21" t="n">
+      <c r="H21" t="n">
         <v>1</v>
       </c>
-      <c r="G21" t="n">
+      <c r="I21" t="n">
         <v>4</v>
       </c>
     </row>
@@ -15696,18 +15866,26 @@
         </is>
       </c>
       <c r="C22" t="n">
+        <v>2255.6</v>
+      </c>
+      <c r="D22" t="n">
         <v>2255.568</v>
       </c>
-      <c r="D22" t="n">
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
         <v>699.2</v>
       </c>
-      <c r="E22" t="n">
+      <c r="G22" t="n">
         <v>31</v>
       </c>
-      <c r="F22" t="n">
+      <c r="H22" t="n">
         <v>2</v>
       </c>
-      <c r="G22" t="n">
+      <c r="I22" t="n">
         <v>6</v>
       </c>
     </row>
@@ -15723,18 +15901,26 @@
         </is>
       </c>
       <c r="C23" t="n">
+        <v>6197</v>
+      </c>
+      <c r="D23" t="n">
         <v>6197.025</v>
       </c>
-      <c r="D23" t="n">
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
         <v>2557.2</v>
       </c>
-      <c r="E23" t="n">
+      <c r="G23" t="n">
         <v>41.3</v>
       </c>
-      <c r="F23" t="n">
+      <c r="H23" t="n">
         <v>1</v>
       </c>
-      <c r="G23" t="n">
+      <c r="I23" t="n">
         <v>5</v>
       </c>
     </row>
@@ -15750,18 +15936,26 @@
         </is>
       </c>
       <c r="C24" t="n">
+        <v>3006.8</v>
+      </c>
+      <c r="D24" t="n">
         <v>3006.756</v>
       </c>
-      <c r="D24" t="n">
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
         <v>2102.3</v>
       </c>
-      <c r="E24" t="n">
+      <c r="G24" t="n">
         <v>69.90000000000001</v>
       </c>
-      <c r="F24" t="n">
+      <c r="H24" t="n">
         <v>1</v>
       </c>
-      <c r="G24" t="n">
+      <c r="I24" t="n">
         <v>2</v>
       </c>
     </row>
@@ -15777,18 +15971,26 @@
         </is>
       </c>
       <c r="C25" t="n">
+        <v>1289.5</v>
+      </c>
+      <c r="D25" t="n">
         <v>1289.543</v>
       </c>
-      <c r="D25" t="n">
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
         <v>201.3</v>
       </c>
-      <c r="E25" t="n">
+      <c r="G25" t="n">
         <v>15.6</v>
       </c>
-      <c r="F25" t="n">
+      <c r="H25" t="n">
         <v>2</v>
       </c>
-      <c r="G25" t="n">
+      <c r="I25" t="n">
         <v>5</v>
       </c>
     </row>
@@ -15804,18 +16006,26 @@
         </is>
       </c>
       <c r="C26" t="n">
+        <v>27266.5</v>
+      </c>
+      <c r="D26" t="n">
         <v>27266.495</v>
       </c>
-      <c r="D26" t="n">
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
         <v>22414.6</v>
       </c>
-      <c r="E26" t="n">
+      <c r="G26" t="n">
         <v>82.2</v>
       </c>
-      <c r="F26" t="n">
+      <c r="H26" t="n">
         <v>4</v>
       </c>
-      <c r="G26" t="n">
+      <c r="I26" t="n">
         <v>8</v>
       </c>
     </row>
@@ -15831,18 +16041,26 @@
         </is>
       </c>
       <c r="C27" t="n">
+        <v>2078</v>
+      </c>
+      <c r="D27" t="n">
         <v>2077.96</v>
       </c>
-      <c r="D27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" t="n">
-        <v>0</v>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
       </c>
       <c r="F27" t="n">
         <v>0</v>
       </c>
       <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
         <v>2</v>
       </c>
     </row>
@@ -15858,18 +16076,26 @@
         </is>
       </c>
       <c r="C28" t="n">
+        <v>3188051.9</v>
+      </c>
+      <c r="D28" t="n">
         <v>3188051.922</v>
       </c>
-      <c r="D28" t="n">
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
         <v>2187.9</v>
       </c>
-      <c r="E28" t="n">
+      <c r="G28" t="n">
         <v>0.1</v>
       </c>
-      <c r="F28" t="n">
+      <c r="H28" t="n">
         <v>1</v>
       </c>
-      <c r="G28" t="n">
+      <c r="I28" t="n">
         <v>17</v>
       </c>
     </row>
@@ -15885,18 +16111,26 @@
         </is>
       </c>
       <c r="C29" t="n">
+        <v>91563.5</v>
+      </c>
+      <c r="D29" t="n">
         <v>91563.489</v>
       </c>
-      <c r="D29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" t="n">
-        <v>0</v>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
       </c>
       <c r="F29" t="n">
         <v>0</v>
       </c>
       <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" t="n">
         <v>2</v>
       </c>
     </row>
@@ -24955,7 +25189,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>improving</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -25743,7 +25977,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>improving</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -25962,7 +26196,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>improving</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -26171,7 +26405,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>improving</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
@@ -26876,7 +27110,7 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>improving</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
@@ -27100,7 +27334,7 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>improving</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
@@ -27606,7 +27840,7 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>improving</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
@@ -28127,7 +28361,7 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>improving</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
@@ -43120,7 +43354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43141,10 +43375,20 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>printed_total</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>total_basis</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>matched_distinct</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -43169,6 +43413,14 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>OK</t>
         </is>
       </c>
@@ -43185,12 +43437,20 @@
         </is>
       </c>
       <c r="C3" t="n">
+        <v>947.5</v>
+      </c>
+      <c r="D3" t="n">
         <v>947.481</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
         <v>0</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43208,12 +43468,20 @@
         </is>
       </c>
       <c r="C4" t="n">
+        <v>32101.8</v>
+      </c>
+      <c r="D4" t="n">
         <v>32101.792</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
         <v>31837.4</v>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43231,12 +43499,20 @@
         </is>
       </c>
       <c r="C5" t="n">
+        <v>92730.7</v>
+      </c>
+      <c r="D5" t="n">
         <v>92730.663</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
         <v>14900.5</v>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43254,12 +43530,20 @@
         </is>
       </c>
       <c r="C6" t="n">
+        <v>16664.3</v>
+      </c>
+      <c r="D6" t="n">
         <v>16664.296</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
         <v>5415.6</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43277,12 +43561,20 @@
         </is>
       </c>
       <c r="C7" t="n">
+        <v>4135.5</v>
+      </c>
+      <c r="D7" t="n">
         <v>4135.507</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
         <v>1125</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43300,12 +43592,20 @@
         </is>
       </c>
       <c r="C8" t="n">
+        <v>278581.5</v>
+      </c>
+      <c r="D8" t="n">
         <v>278581.467</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
         <v>277724.3</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43323,12 +43623,20 @@
         </is>
       </c>
       <c r="C9" t="n">
+        <v>1002681.6</v>
+      </c>
+      <c r="D9" t="n">
         <v>1002681.586</v>
       </c>
-      <c r="D9" t="n">
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
         <v>886652.4</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43346,12 +43654,20 @@
         </is>
       </c>
       <c r="C10" t="n">
+        <v>219826.8</v>
+      </c>
+      <c r="D10" t="n">
         <v>219826.755</v>
       </c>
-      <c r="D10" t="n">
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
         <v>208505.3</v>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43369,12 +43685,20 @@
         </is>
       </c>
       <c r="C11" t="n">
+        <v>107634.1</v>
+      </c>
+      <c r="D11" t="n">
         <v>107634.125</v>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
         <v>78626.2</v>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43392,12 +43716,20 @@
         </is>
       </c>
       <c r="C12" t="n">
+        <v>162614</v>
+      </c>
+      <c r="D12" t="n">
         <v>162614.024</v>
       </c>
-      <c r="D12" t="n">
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
         <v>86971.7</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43415,12 +43747,20 @@
         </is>
       </c>
       <c r="C13" t="n">
+        <v>2877.3</v>
+      </c>
+      <c r="D13" t="n">
         <v>2877.345</v>
       </c>
-      <c r="D13" t="n">
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
         <v>2026.6</v>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43438,12 +43778,20 @@
         </is>
       </c>
       <c r="C14" t="n">
+        <v>2170.6</v>
+      </c>
+      <c r="D14" t="n">
         <v>2170.599</v>
       </c>
-      <c r="D14" t="n">
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
         <v>1412.4</v>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43461,12 +43809,20 @@
         </is>
       </c>
       <c r="C15" t="n">
+        <v>10239.4</v>
+      </c>
+      <c r="D15" t="n">
         <v>10239.386</v>
       </c>
-      <c r="D15" t="n">
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
         <v>9046.700000000001</v>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43484,12 +43840,20 @@
         </is>
       </c>
       <c r="C16" t="n">
+        <v>682.6</v>
+      </c>
+      <c r="D16" t="n">
         <v>682.617</v>
       </c>
-      <c r="D16" t="n">
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
         <v>682.6</v>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43507,12 +43871,20 @@
         </is>
       </c>
       <c r="C17" t="n">
+        <v>2937.2</v>
+      </c>
+      <c r="D17" t="n">
         <v>2937.235</v>
       </c>
-      <c r="D17" t="n">
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
         <v>2495.5</v>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43530,12 +43902,20 @@
         </is>
       </c>
       <c r="C18" t="n">
+        <v>15386.2</v>
+      </c>
+      <c r="D18" t="n">
         <v>15386.176</v>
       </c>
-      <c r="D18" t="n">
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
         <v>13557.4</v>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43553,12 +43933,20 @@
         </is>
       </c>
       <c r="C19" t="n">
+        <v>17427.2</v>
+      </c>
+      <c r="D19" t="n">
         <v>17427.157</v>
       </c>
-      <c r="D19" t="n">
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
         <v>6203.7</v>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43576,12 +43964,20 @@
         </is>
       </c>
       <c r="C20" t="n">
+        <v>29160.4</v>
+      </c>
+      <c r="D20" t="n">
         <v>29160.377</v>
       </c>
-      <c r="D20" t="n">
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
         <v>23107.1</v>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43599,12 +43995,20 @@
         </is>
       </c>
       <c r="C21" t="n">
+        <v>3304.9</v>
+      </c>
+      <c r="D21" t="n">
         <v>3304.874</v>
       </c>
-      <c r="D21" t="n">
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
         <v>592.4</v>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43622,12 +44026,20 @@
         </is>
       </c>
       <c r="C22" t="n">
+        <v>2255.6</v>
+      </c>
+      <c r="D22" t="n">
         <v>2255.568</v>
       </c>
-      <c r="D22" t="n">
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
         <v>699.2</v>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43645,12 +44057,20 @@
         </is>
       </c>
       <c r="C23" t="n">
+        <v>6197</v>
+      </c>
+      <c r="D23" t="n">
         <v>6197.025</v>
       </c>
-      <c r="D23" t="n">
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
         <v>2557.2</v>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43668,12 +44088,20 @@
         </is>
       </c>
       <c r="C24" t="n">
+        <v>3006.8</v>
+      </c>
+      <c r="D24" t="n">
         <v>3006.756</v>
       </c>
-      <c r="D24" t="n">
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
         <v>2102.3</v>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43691,12 +44119,20 @@
         </is>
       </c>
       <c r="C25" t="n">
+        <v>1289.5</v>
+      </c>
+      <c r="D25" t="n">
         <v>1289.543</v>
       </c>
-      <c r="D25" t="n">
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
         <v>201.3</v>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43714,12 +44150,20 @@
         </is>
       </c>
       <c r="C26" t="n">
+        <v>27266.5</v>
+      </c>
+      <c r="D26" t="n">
         <v>27266.495</v>
       </c>
-      <c r="D26" t="n">
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
         <v>22414.6</v>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43737,12 +44181,20 @@
         </is>
       </c>
       <c r="C27" t="n">
+        <v>2078</v>
+      </c>
+      <c r="D27" t="n">
         <v>2077.96</v>
       </c>
-      <c r="D27" t="n">
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
         <v>0</v>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43760,12 +44212,20 @@
         </is>
       </c>
       <c r="C28" t="n">
+        <v>3188051.9</v>
+      </c>
+      <c r="D28" t="n">
         <v>3188051.922</v>
       </c>
-      <c r="D28" t="n">
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
         <v>2187.9</v>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -43783,12 +44243,20 @@
         </is>
       </c>
       <c r="C29" t="n">
+        <v>91563.5</v>
+      </c>
+      <c r="D29" t="n">
         <v>91563.489</v>
       </c>
-      <c r="D29" t="n">
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>printed</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
         <v>0</v>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>OK</t>
         </is>

</xml_diff>